<commit_message>
commit by chirag , integrate uni uni
</commit_message>
<xml_diff>
--- a/Documents/DTDC-DPD Service types & codes - Online booking 2026.xlsx
+++ b/Documents/DTDC-DPD Service types & codes - Online booking 2026.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="64">
   <si>
     <t xml:space="preserve">Weight</t>
   </si>
@@ -61,6 +61,9 @@
     <t xml:space="preserve">DPD112</t>
   </si>
   <si>
+    <t xml:space="preserve">in use</t>
+  </si>
+  <si>
     <t xml:space="preserve">10 to 20 kgs</t>
   </si>
   <si>
@@ -74,6 +77,9 @@
   </si>
   <si>
     <t xml:space="preserve">MDPD112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">only for multiple shipment</t>
   </si>
   <si>
     <t xml:space="preserve">0.1- 30 Kgs</t>
@@ -458,32 +464,36 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -491,95 +501,95 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -667,9 +677,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>2653560</xdr:colOff>
+      <xdr:colOff>2653200</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>31680</xdr:rowOff>
+      <xdr:rowOff>31320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -683,7 +693,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3107880" y="1530720"/>
-          <a:ext cx="5842440" cy="365400"/>
+          <a:ext cx="5842080" cy="365040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -705,9 +715,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1377360</xdr:colOff>
+      <xdr:colOff>1377000</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>144360</xdr:rowOff>
+      <xdr:rowOff>144000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -721,7 +731,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="4361400" cy="1103760"/>
+          <a:ext cx="4361040" cy="1103400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -914,418 +924,434 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C3:F46"/>
+  <dimension ref="C3:H46"/>
   <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="33.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="33.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.79"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="F14" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="F15" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="F16" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="10" t="s">
         <v>7</v>
       </c>
+      <c r="G17" s="0" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="7" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E19" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F19" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="0" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C21" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C23" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C24" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C26" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C29" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F29" s="18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C31" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F31" s="18" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C34" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C35" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C38" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C39" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C40" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C43" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D43" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="E43" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="F43" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C44" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D44" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E44" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="F44" s="30" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" s="17" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="F29" s="17" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E30" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="F30" s="17" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="E31" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E32" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="F32" s="20" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="F34" s="22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="D35" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="E35" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="F35" s="25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C39" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="F39" s="17" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C40" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="E40" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="F40" s="20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C43" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D43" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="E43" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="F43" s="22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C44" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="D44" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="E44" s="28" t="s">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C45" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="F44" s="29" t="s">
+      <c r="D45" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="E45" s="29" t="s">
+        <v>60</v>
+      </c>
+      <c r="F45" s="30" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C45" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="D45" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="E45" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="F45" s="29" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C46" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="D46" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="E46" s="28" t="s">
+      <c r="C46" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="F46" s="29" t="s">
+      <c r="D46" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="E46" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" s="30" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>